<commit_message>
feat(core): add configurable safeDiv guards
</commit_message>
<xml_diff>
--- a/packages/examples/showcase/native-excel-forecast-table/artifact/native-excel-forecast-table.xlsx
+++ b/packages/examples/showcase/native-excel-forecast-table/artifact/native-excel-forecast-table.xlsx
@@ -244,22 +244,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ForecastTable" displayName="ForecastTable" ref="A1:G12" totalsRowCount="1" headerRowCount="1">
-  <autoFilter ref="A1:G11"/>
-  <tableColumns count="7">
-    <tableColumn id="1" name="Rep" totalsRowLabel="TOTAL"/>
-    <tableColumn id="2" name="Territory"/>
-    <tableColumn id="3" name="Stage"/>
-    <tableColumn id="4" name="Units" totalsRowFunction="sum"/>
-    <tableColumn id="5" name="Revenue" totalsRowFunction="sum"/>
-    <tableColumn id="6" name="Avg Price" totalsRowLabel="-">
-      <calculatedColumnFormula>ROUND((ForecastTable[@[Revenue]]/ForecastTable[@[Units]]),2)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="7" name="Close Month" totalsRowFunction="max"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?><table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ForecastTable" displayName="ForecastTable" ref="A1:G12" totalsRowCount="1" headerRowCount="1"><autoFilter ref="A1:G11"/><tableColumns count="7"><tableColumn id="1" name="Rep" totalsRowLabel="TOTAL"/><tableColumn id="2" name="Territory"/><tableColumn id="3" name="Stage"/><tableColumn id="4" name="Units" totalsRowFunction="sum"/><tableColumn id="5" name="Revenue" totalsRowFunction="sum"/><tableColumn id="6" name="Avg Price" totalsRowLabel="-"><calculatedColumnFormula>ROUND(IF((ForecastTable[@[Units]]<>0),(ForecastTable[@[Revenue]]/ForecastTable[@[Units]]),0),2)</calculatedColumnFormula></tableColumn><tableColumn id="7" name="Close Month" totalsRowFunction="max"/></tableColumns><tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/></table>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -316,7 +301,7 @@
         <v>307415</v>
       </c>
       <c r="F2" s="5">
-        <f>ROUND(([@[Revenue]]/[@[Units]]),2)</f>
+        <f>ROUND(IF(([@[Units]]&lt;&gt;0),([@[Revenue]]/[@[Units]]),0),2)</f>
       </c>
       <c r="G2" s="2" t="s">
         <v>10</v>
@@ -339,7 +324,7 @@
         <v>185220</v>
       </c>
       <c r="F3" s="5">
-        <f>ROUND(([@[Revenue]]/[@[Units]]),2)</f>
+        <f>ROUND(IF(([@[Units]]&lt;&gt;0),([@[Revenue]]/[@[Units]]),0),2)</f>
       </c>
       <c r="G3" s="2" t="s">
         <v>14</v>
@@ -362,7 +347,7 @@
         <v>396734</v>
       </c>
       <c r="F4" s="5">
-        <f>ROUND(([@[Revenue]]/[@[Units]]),2)</f>
+        <f>ROUND(IF(([@[Units]]&lt;&gt;0),([@[Revenue]]/[@[Units]]),0),2)</f>
       </c>
       <c r="G4" s="2" t="s">
         <v>18</v>
@@ -385,7 +370,7 @@
         <v>356112</v>
       </c>
       <c r="F5" s="5">
-        <f>ROUND(([@[Revenue]]/[@[Units]]),2)</f>
+        <f>ROUND(IF(([@[Units]]&lt;&gt;0),([@[Revenue]]/[@[Units]]),0),2)</f>
       </c>
       <c r="G5" s="2" t="s">
         <v>14</v>
@@ -408,7 +393,7 @@
         <v>325532</v>
       </c>
       <c r="F6" s="5">
-        <f>ROUND(([@[Revenue]]/[@[Units]]),2)</f>
+        <f>ROUND(IF(([@[Units]]&lt;&gt;0),([@[Revenue]]/[@[Units]]),0),2)</f>
       </c>
       <c r="G6" s="2" t="s">
         <v>14</v>
@@ -431,7 +416,7 @@
         <v>181200</v>
       </c>
       <c r="F7" s="5">
-        <f>ROUND(([@[Revenue]]/[@[Units]]),2)</f>
+        <f>ROUND(IF(([@[Units]]&lt;&gt;0),([@[Revenue]]/[@[Units]]),0),2)</f>
       </c>
       <c r="G7" s="2" t="s">
         <v>14</v>
@@ -454,7 +439,7 @@
         <v>218137</v>
       </c>
       <c r="F8" s="5">
-        <f>ROUND(([@[Revenue]]/[@[Units]]),2)</f>
+        <f>ROUND(IF(([@[Units]]&lt;&gt;0),([@[Revenue]]/[@[Units]]),0),2)</f>
       </c>
       <c r="G8" s="2" t="s">
         <v>27</v>
@@ -477,7 +462,7 @@
         <v>181799</v>
       </c>
       <c r="F9" s="5">
-        <f>ROUND(([@[Revenue]]/[@[Units]]),2)</f>
+        <f>ROUND(IF(([@[Units]]&lt;&gt;0),([@[Revenue]]/[@[Units]]),0),2)</f>
       </c>
       <c r="G9" s="2" t="s">
         <v>14</v>
@@ -500,7 +485,7 @@
         <v>93641</v>
       </c>
       <c r="F10" s="5">
-        <f>ROUND(([@[Revenue]]/[@[Units]]),2)</f>
+        <f>ROUND(IF(([@[Units]]&lt;&gt;0),([@[Revenue]]/[@[Units]]),0),2)</f>
       </c>
       <c r="G10" s="2" t="s">
         <v>10</v>
@@ -523,7 +508,7 @@
         <v>160048</v>
       </c>
       <c r="F11" s="5">
-        <f>ROUND(([@[Revenue]]/[@[Units]]),2)</f>
+        <f>ROUND(IF(([@[Units]]&lt;&gt;0),([@[Revenue]]/[@[Units]]),0),2)</f>
       </c>
       <c r="G11" s="2" t="s">
         <v>14</v>

</xml_diff>